<commit_message>
Add latest data updates (DB and medicine export)
</commit_message>
<xml_diff>
--- a/medicine_list.xlsx
+++ b/medicine_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H156"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2813,21 +2813,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MONJARO 5 MG KWIK PEN</t>
+          <t>MONJARO 2.5 MG KWIK PEN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>D919450</t>
+          <t>D924668</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>05/2027</t>
+          <t>01/2027</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>16406.25</v>
+        <v>13125</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
@@ -2854,12 +2854,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>D928027</t>
+          <t>D919450</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>05/2027</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2885,60 +2885,60 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MOX-CV-625</t>
+          <t>MONJARO 5 MG KWIK PEN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BYC0051</t>
+          <t>D928027</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>01/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>19.53</v>
+        <v>16406.25</v>
       </c>
       <c r="E69" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G69" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Unit of 1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NAXDOM-500</t>
+          <t>MOX-CV-625</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>FHC0946</t>
+          <t>BYC0051</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>09/2028</t>
+          <t>01/2027</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>11.75</v>
+        <v>19.53</v>
       </c>
       <c r="E70" t="n">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2946,75 +2946,75 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NEOGADINE ELIXIR SYP</t>
+          <t>NAXDOM-500</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>B02K25098</t>
+          <t>FHC0946</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>01/2027</t>
+          <t>09/2028</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>233.5</v>
+        <v>11.75</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Bottle of 1</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NOVOFINE NEEDLE</t>
+          <t>NEOGADINE ELIXIR SYP</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>544N</t>
+          <t>B02K25098</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>09/2030</t>
+          <t>01/2027</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>14</v>
+        <v>233.5</v>
       </c>
       <c r="E72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Bottle</t>
         </is>
       </c>
       <c r="G72" t="n">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Unit of 1</t>
+          <t>Bottle of 1</t>
         </is>
       </c>
     </row>
@@ -3034,19 +3034,19 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>317B</t>
+          <t>544N</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>03/2028</t>
+          <t>09/2030</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>13.13</v>
+        <v>14</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3070,19 +3070,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>523F</t>
+          <t>317B</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>05/2030</t>
+          <t>03/2028</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>14</v>
+        <v>13.13</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3106,16 +3106,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>012477</t>
+          <t>523F</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>05/2029</t>
+          <t>05/2030</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6.09</v>
+        <v>14</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
@@ -3137,36 +3137,36 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NUROKIND-LC</t>
+          <t>NOVOFINE NEEDLE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>B95Y132</t>
+          <t>012477</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>05/2029</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>15.927</v>
+        <v>6.09</v>
       </c>
       <c r="E76" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G76" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Unit of 1</t>
         </is>
       </c>
     </row>
@@ -3178,19 +3178,19 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>B95Y125</t>
+          <t>B95Y132</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D77" t="n">
         <v>15.927</v>
       </c>
       <c r="E77" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>B95Y128</t>
+          <t>B95Y125</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3245,24 +3245,24 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>OLKEM 20</t>
+          <t>NUROKIND-LC</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25443043</t>
+          <t>B95Y128</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>22.78</v>
+        <v>15.927</v>
       </c>
       <c r="E79" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3270,11 +3270,11 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
@@ -3286,19 +3286,19 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>25444565</t>
+          <t>25443043</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>11/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>15.186</v>
+        <v>22.78</v>
       </c>
       <c r="E80" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -3306,35 +3306,35 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>OLKEM AM 20</t>
+          <t>OLKEM 20</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>25490463</t>
+          <t>25444565</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>04/2027</t>
+          <t>11/2027</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>27.42</v>
+        <v>15.186</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>300</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3342,11 +3342,11 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
@@ -3358,19 +3358,19 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25490707</t>
+          <t>25490463</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>04/2027</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>27.42</v>
       </c>
       <c r="E82" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3389,24 +3389,24 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>OLKEM TRIO 6.25</t>
+          <t>OLKEM AM 20</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>OTS25008SS</t>
+          <t>25490707</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>19.59</v>
+        <v>27.42</v>
       </c>
       <c r="E83" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3425,24 +3425,24 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>OLMEZEST 20</t>
+          <t>OLKEM TRIO 6.25</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SIG899C</t>
+          <t>OTS25008SS</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>02/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>15</v>
+        <v>19.59</v>
       </c>
       <c r="E84" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3461,24 +3461,24 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>OLMEZEST AM</t>
+          <t>OLMEZEST 20</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SIG1951A</t>
+          <t>SIG899C</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>02/2027</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>19.5</v>
+        <v>15</v>
       </c>
       <c r="E85" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3497,24 +3497,24 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ONDEM-MD-4MG</t>
+          <t>OLMEZEST AM</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25442254</t>
+          <t>SIG1951A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>05/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>5.48</v>
+        <v>19.5</v>
       </c>
       <c r="E86" t="n">
-        <v>360</v>
+        <v>100</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3533,24 +3533,24 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ONDERO D10</t>
+          <t>ONDEM-MD-4MG</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EMV252581A</t>
+          <t>25442254</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>05/2027</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>22.12</v>
+        <v>5.48</v>
       </c>
       <c r="E87" t="n">
-        <v>100</v>
+        <v>360</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3569,24 +3569,24 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ONDERO DM 500</t>
+          <t>ONDERO D10</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>GT251469</t>
+          <t>EMV252581A</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>21.55</v>
+        <v>22.12</v>
       </c>
       <c r="E88" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3605,24 +3605,24 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>OVRAL-L TAB</t>
+          <t>ONDERO DM 500</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MR6546</t>
+          <t>GT251469</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>01/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>3.221</v>
+        <v>21.55</v>
       </c>
       <c r="E89" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3630,35 +3630,35 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Strip of 21</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>OXRAMET S XR 10/100/500</t>
+          <t>OVRAL-L TAB</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>GTG3150A</t>
+          <t>MR6546</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>01/2027</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>22.294</v>
+        <v>3.221</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3666,11 +3666,11 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Strip of 7</t>
+          <t>Strip of 21</t>
         </is>
       </c>
     </row>
@@ -3682,19 +3682,19 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>GTG3613A</t>
+          <t>GTG3150A</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>21.294</v>
+        <v>22.294</v>
       </c>
       <c r="E91" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3713,60 +3713,60 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>OZEMPIC 0.25 MG PEN</t>
+          <t>OXRAMET S XR 10/100/500</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>RP5V726</t>
+          <t>GTG3613A</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>07/2028</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>8800</v>
+        <v>21.294</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Unit of 1</t>
+          <t>Strip of 7</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PEN NEEDLE</t>
+          <t>OZEMPIC 0.25 MG PEN</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>5056002</t>
+          <t>RP5V726</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>02/2030</t>
+          <t>07/2028</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>20.25</v>
+        <v>8800</v>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3785,96 +3785,96 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PIOZ 15MG TAB</t>
+          <t>PEN NEEDLE</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>48020714</t>
+          <t>5056002</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>02/2030</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>78.52</v>
+        <v>20.25</v>
       </c>
       <c r="E94" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G94" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Unit of 1</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PIOZ MF-15 TAB</t>
+          <t>PEN NEEDLE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>28027440</t>
+          <t>317B</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>01/2028</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>14.592</v>
+        <v>13.13</v>
       </c>
       <c r="E95" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G95" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Unit of 4</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ROSUVAS 10</t>
+          <t>PIOZ 15MG TAB</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SIG1644A</t>
+          <t>48020714</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>01/2028</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>23.062</v>
+        <v>78.52</v>
       </c>
       <c r="E96" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -3882,35 +3882,35 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ROSUVAS 5</t>
+          <t>PIOZ MF-15 TAB</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SIG1784A</t>
+          <t>28027440</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>01/2028</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>13.125</v>
+        <v>14.592</v>
       </c>
       <c r="E97" t="n">
-        <v>30</v>
+        <v>160</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -3918,35 +3918,35 @@
         </is>
       </c>
       <c r="G97" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SHELCAL-500</t>
+          <t>ROSUVAS 10</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>8LV2M362</t>
+          <t>SIG1644A</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>01/2028</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>9.91</v>
+        <v>23.062</v>
       </c>
       <c r="E98" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -3965,24 +3965,24 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SHELCAL-500</t>
+          <t>ROSUVAS 5</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>8LV2M447</t>
+          <t>SIG1784A</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>01/2028</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>10.89</v>
+        <v>13.125</v>
       </c>
       <c r="E99" t="n">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4006,16 +4006,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>8LVM349</t>
+          <t>8LV2M362</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>9.912000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="E100" t="n">
         <v>0</v>
@@ -4037,24 +4037,24 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SHELCAL-CT</t>
+          <t>SHELCAL-500</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>GAXF0023</t>
+          <t>8LV2M447</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>25.28</v>
+        <v>10.89</v>
       </c>
       <c r="E101" t="n">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4073,24 +4073,24 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SHELCAL-XT</t>
+          <t>SHELCAL-500</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2SG6M104</t>
+          <t>8LVM349</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>26.81</v>
+        <v>9.912000000000001</v>
       </c>
       <c r="E102" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -4109,24 +4109,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SITARA M 100\500</t>
+          <t>SHELCAL-CT</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EMV252758C</t>
+          <t>GAXF0023</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>16.383</v>
+        <v>25.28</v>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -4134,23 +4134,23 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SITARA M 100\500</t>
+          <t>SHELCAL-XT</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EMV252762</t>
+          <t>2SG6M104</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4159,10 +4159,10 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>16.383</v>
+        <v>26.81</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -4170,35 +4170,35 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SITARA M 50/500</t>
+          <t>SITARA M 100\500</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EMV252263</t>
+          <t>EMV252758C</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>18.422</v>
+        <v>16.383</v>
       </c>
       <c r="E105" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -4217,21 +4217,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SITARED M 50/500</t>
+          <t>SITARA M 100\500</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SIG2194A</t>
+          <t>EMV252762</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>11.75</v>
+        <v>16.383</v>
       </c>
       <c r="E106" t="n">
         <v>0</v>
@@ -4242,35 +4242,35 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SITARED M 50/500</t>
+          <t>SITARA M 50/500</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SIG2272B</t>
+          <t>EMV252263</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11.75</v>
+        <v>18.422</v>
       </c>
       <c r="E107" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4278,35 +4278,35 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SITARED M XR 100/1000</t>
+          <t>SITARED M 50/500</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>GTF1664B</t>
+          <t>SIG2194A</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>14.906</v>
+        <v>11.75</v>
       </c>
       <c r="E108" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -4314,35 +4314,35 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SITARED M XR 100/500</t>
+          <t>SITARED M 50/500</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>AXC0097</t>
+          <t>SIG2272B</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>13.5</v>
+        <v>11.75</v>
       </c>
       <c r="E109" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -4361,24 +4361,24 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SPORLAC-DS</t>
+          <t>SITARED M XR 100/1000</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>BDS25019</t>
+          <t>GTF1664B</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>8.965999999999999</v>
+        <v>14.906</v>
       </c>
       <c r="E110" t="n">
-        <v>600</v>
+        <v>20</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4386,35 +4386,35 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Strip of 25</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>STEMETIL-MD TAB</t>
+          <t>SITARED M XR 100/500</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>SEA25022</t>
+          <t>AXC0097</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>11.87</v>
+        <v>13.5</v>
       </c>
       <c r="E111" t="n">
-        <v>279</v>
+        <v>90</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4433,24 +4433,24 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SYSCAN-150</t>
+          <t>SPORLAC-DS</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>CBD2M001</t>
+          <t>BDS25019</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>01/2028</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>20.17</v>
+        <v>8.965999999999999</v>
       </c>
       <c r="E112" t="n">
-        <v>2</v>
+        <v>600</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -4458,71 +4458,71 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Strip of 1</t>
+          <t>Strip of 25</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>T-BACT OINT 5GM</t>
+          <t>STEMETIL-MD TAB</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>K73K</t>
+          <t>SEA25022</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>108.36</v>
+        <v>11.87</v>
       </c>
       <c r="E113" t="n">
-        <v>5</v>
+        <v>279</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Tube</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Tube of 1</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>TELMEKIND-TRIO 6.25 TAB</t>
+          <t>SYSCAN-150</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>A6OAY022</t>
+          <t>CBD2M001</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>01/2028</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>12.454</v>
+        <v>20.17</v>
       </c>
       <c r="E114" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -4530,119 +4530,119 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Strip of 1</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>TELVOK-40 MG</t>
+          <t>T-BACT OINT 5GM</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>ATH2511142</t>
+          <t>K73K</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>7.097</v>
+        <v>108.36</v>
       </c>
       <c r="E115" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Tube</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Tube of 1</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>THYRONORM 100</t>
+          <t>TELMEKIND-TRIO 6.25 TAB</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TMH25237</t>
+          <t>A6OAY022</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>168.82</v>
+        <v>12.454</v>
       </c>
       <c r="E116" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Bottle of 1</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>THYRONORM 100</t>
+          <t>TELVOK-40 MG</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TMN25217</t>
+          <t>ATH2511142</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>168.82</v>
+        <v>7.097</v>
       </c>
       <c r="E117" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Bottle of 1</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
@@ -4654,19 +4654,19 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>TMH25258</t>
+          <t>TMH25237</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D118" t="n">
         <v>168.82</v>
       </c>
       <c r="E118" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -4685,21 +4685,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>THYRONORM 112</t>
+          <t>THYRONORM 100</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>TMI25008*</t>
+          <t>TMN25217</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>212.72</v>
+        <v>168.82</v>
       </c>
       <c r="E119" t="n">
         <v>0</v>
@@ -4721,12 +4721,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>THYRONORM 112</t>
+          <t>THYRONORM 100</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EBRH5005</t>
+          <t>TMH25258</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -4735,10 +4735,10 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>251.7</v>
+        <v>168.82</v>
       </c>
       <c r="E120" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -4757,21 +4757,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>THYRONORM 12.5</t>
+          <t>THYRONORM 112</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>AEL0406*</t>
+          <t>TMI25008*</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>189.72</v>
+        <v>212.72</v>
       </c>
       <c r="E121" t="n">
         <v>0</v>
@@ -4793,24 +4793,24 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>THYRONORM 12.5</t>
+          <t>THYRONORM 112</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>AEL0477</t>
+          <t>EBRH5005</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>11/2027</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>189.72</v>
+        <v>251.7</v>
       </c>
       <c r="E122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -4829,21 +4829,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>THYRONORM 125</t>
+          <t>THYRONORM 12.5</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EBRI5008</t>
+          <t>AEL0406*</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>216.63</v>
+        <v>189.72</v>
       </c>
       <c r="E123" t="n">
         <v>0</v>
@@ -4865,24 +4865,24 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>THYRONORM 125</t>
+          <t>THYRONORM 12.5</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>EBRI5023</t>
+          <t>AEL0477</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>216.63</v>
+        <v>189.72</v>
       </c>
       <c r="E124" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -4901,21 +4901,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>THYRONORM 25</t>
+          <t>THYRONORM 125</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TMB25278</t>
+          <t>EBRI5008</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>185.4</v>
+        <v>216.63</v>
       </c>
       <c r="E125" t="n">
         <v>0</v>
@@ -4937,12 +4937,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>THYRONORM 25</t>
+          <t>THYRONORM 125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TMB25292</t>
+          <t>EBRI5023</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -4951,10 +4951,10 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>185.4</v>
+        <v>216.63</v>
       </c>
       <c r="E126" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>THYRONORM 37.5</t>
+          <t>THYRONORM 25</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TMC25063*</t>
+          <t>TMB25278</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>187.85</v>
+        <v>185.4</v>
       </c>
       <c r="E127" t="n">
         <v>0</v>
@@ -5009,12 +5009,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>THYRONORM 50</t>
+          <t>THYRONORM 25</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>TMD25396*</t>
+          <t>TMB25292</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5023,10 +5023,10 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>132.02</v>
+        <v>185.4</v>
       </c>
       <c r="E128" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -5045,24 +5045,24 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>THYRONORM 50</t>
+          <t>THYRONORM 37.5</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TMD25396</t>
+          <t>TMC25063*</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>132.02</v>
+        <v>187.85</v>
       </c>
       <c r="E129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -5081,24 +5081,24 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>THYRONORM 62.5</t>
+          <t>THYRONORM 50</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EBRG5028*</t>
+          <t>TMD25396*</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>206.37</v>
+        <v>132.02</v>
       </c>
       <c r="E130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -5117,24 +5117,24 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>THYRONORM 62.5</t>
+          <t>THYRONORM 50</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EBRF5036</t>
+          <t>TMD25396</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>206.37</v>
+        <v>132.02</v>
       </c>
       <c r="E131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -5153,12 +5153,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>THYRONORM 75</t>
+          <t>THYRONORM 62.5</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TMF25182*</t>
+          <t>EBRG5028*</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5167,10 +5167,10 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>183.97</v>
+        <v>206.37</v>
       </c>
       <c r="E132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -5189,24 +5189,24 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>THYRONORM 75</t>
+          <t>THYRONORM 62.5</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TMF25231</t>
+          <t>EBRF5036</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>183.97</v>
+        <v>206.37</v>
       </c>
       <c r="E133" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -5230,12 +5230,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TMF25209</t>
+          <t>TMF25182*</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -5261,21 +5261,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>THYRONORM 88</t>
+          <t>THYRONORM 75</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>EBRG5028*</t>
+          <t>TMF25231</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>211.27</v>
+        <v>183.97</v>
       </c>
       <c r="E135" t="n">
         <v>0</v>
@@ -5297,24 +5297,24 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>THYRONORM 88</t>
+          <t>THYRONORM 75</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EBRG5036</t>
+          <t>TMF25209</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>211.28</v>
+        <v>183.97</v>
       </c>
       <c r="E136" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -5333,96 +5333,96 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TRIGLYNASE-1</t>
+          <t>THYRONORM 88</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>28027170</t>
+          <t>EBRG5028*</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>02/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>6.422</v>
+        <v>211.27</v>
       </c>
       <c r="E137" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Bottle</t>
         </is>
       </c>
       <c r="G137" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Bottle of 1</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>TRIGLYNASE-2</t>
+          <t>THYRONORM 88</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>28027385</t>
+          <t>EBRG5036</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>04/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>9.352</v>
+        <v>211.28</v>
       </c>
       <c r="E138" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Bottle</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Bottle of 1</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>TRIGLYNASE-2</t>
+          <t>TRIGLYNASE-1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>28027306</t>
+          <t>28027170</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>03/2027</t>
+          <t>02/2027</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>9.352</v>
+        <v>6.422</v>
       </c>
       <c r="E139" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -5441,24 +5441,24 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>TRIOLMEZEST 40 MG</t>
+          <t>TRIGLYNASE-2</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>GTC2880A</t>
+          <t>28027385</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>04/2027</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>21.844</v>
+        <v>9.352</v>
       </c>
       <c r="E140" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -5477,24 +5477,24 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>TRYPTOMER-10 MG</t>
+          <t>TRIGLYNASE-2</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>D2500387</t>
+          <t>28027306</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10/2027</t>
+          <t>03/2027</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>2.546</v>
+        <v>9.352</v>
       </c>
       <c r="E141" t="n">
-        <v>595</v>
+        <v>0</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -5502,35 +5502,35 @@
         </is>
       </c>
       <c r="G141" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Strip of 30</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>VSL 3 CAP</t>
+          <t>TRIOLMEZEST 40 MG</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>JMG1096A</t>
+          <t>GTC2880A</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>08/2027</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>45.51</v>
+        <v>21.844</v>
       </c>
       <c r="E142" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -5549,24 +5549,24 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>WONRIDE-M1</t>
+          <t>TRYPTOMER-10 MG</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>WNM1325004</t>
+          <t>D2500387</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>07/2027</t>
+          <t>10/2027</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>7.562</v>
+        <v>2.546</v>
       </c>
       <c r="E143" t="n">
-        <v>45</v>
+        <v>595</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -5574,35 +5574,35 @@
         </is>
       </c>
       <c r="G143" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 30</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>WONRIDE-M1</t>
+          <t>VSL 3 CAP</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>WNM1325005</t>
+          <t>JMG1096A</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>11/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>7.562</v>
+        <v>45.51</v>
       </c>
       <c r="E144" t="n">
-        <v>180</v>
+        <v>20</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
@@ -5610,35 +5610,35 @@
         </is>
       </c>
       <c r="G144" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Strip of 15</t>
+          <t>Strip of 10</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>WONRIDE-M2</t>
+          <t>WONRIDE-M1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>WOH25004</t>
+          <t>WNM1325004</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>07/2027</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>8.593999999999999</v>
+        <v>7.562</v>
       </c>
       <c r="E145" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -5657,12 +5657,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>WONRIDE-M2</t>
+          <t>WONRIDE-M1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>WOH25005</t>
+          <t>WNM1325005</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -5671,7 +5671,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>8.593999999999999</v>
+        <v>7.562</v>
       </c>
       <c r="E146" t="n">
         <v>180</v>
@@ -5693,96 +5693,96 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>XGLAR CART</t>
+          <t>WONRIDE-M2</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>C241GH4010</t>
+          <t>WOH25004</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>06/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>640.8</v>
+        <v>8.593999999999999</v>
       </c>
       <c r="E147" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G147" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Unit of 1</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>XSULIN R CART</t>
+          <t>WONRIDE-M2</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TBB030225</t>
+          <t>WOH25005</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>01/2028</t>
+          <t>11/2027</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>175.1</v>
+        <v>8.593999999999999</v>
       </c>
       <c r="E148" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Strip</t>
         </is>
       </c>
       <c r="G148" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Unit of 1</t>
+          <t>Strip of 15</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>XSULIN R CART</t>
+          <t>XGLAR CART</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>A042517604</t>
+          <t>C241GH4010</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>07/2028</t>
+          <t>06/2027</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>375.1</v>
+        <v>640.8</v>
       </c>
       <c r="E149" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -5801,24 +5801,24 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>XSULIN R VIAL</t>
+          <t>XSULIN R CART</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>A032515016</t>
+          <t>TBB030225</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>04/2027</t>
+          <t>01/2028</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>181.39</v>
+        <v>175.1</v>
       </c>
       <c r="E150" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
@@ -5837,24 +5837,24 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>YURPEAK 2.5MG/0.6ML PEN</t>
+          <t>XSULIN R CART</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>D921081</t>
+          <t>A042517604</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>05/2027</t>
+          <t>07/2028</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>13125</v>
+        <v>375.1</v>
       </c>
       <c r="E151" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
@@ -5873,28 +5873,28 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ZEDEX-SF COUGH SYP</t>
+          <t>XSULIN R VIAL</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>D250569</t>
+          <t>A032515016</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>04/2027</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>190.31</v>
+        <v>181.39</v>
       </c>
       <c r="E152" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G152" t="n">
@@ -5902,35 +5902,35 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>Bottle of 1</t>
+          <t>Unit of 1</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ZEDEX-SF COUGH SYP</t>
+          <t>YURPEAK 2.5MG/0.6ML PEN</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>D250570</t>
+          <t>D921081</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>09/2027</t>
+          <t>05/2027</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>190.31</v>
+        <v>13125</v>
       </c>
       <c r="E153" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G153" t="n">
@@ -5938,113 +5938,185 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Bottle of 1</t>
+          <t>Unit of 1</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ZERODOL-P</t>
+          <t>ZEDEX-SF COUGH SYP</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>KVB012511</t>
+          <t>D250569</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>08/2027</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>7.59</v>
+        <v>190.31</v>
       </c>
       <c r="E154" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Bottle</t>
         </is>
       </c>
       <c r="G154" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Bottle of 1</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ZERODOL-SP</t>
+          <t>ZEDEX-SF COUGH SYP</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>FND082504</t>
+          <t>D250570</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>03/2028</t>
+          <t>09/2027</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>13.96</v>
+        <v>190.31</v>
       </c>
       <c r="E155" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Strip</t>
+          <t>Bottle</t>
         </is>
       </c>
       <c r="G155" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Strip of 10</t>
+          <t>Bottle of 1</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
+          <t>ZERODOL-P</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>KVB012511</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>08/2027</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="E156" t="n">
+        <v>50</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>10</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Strip of 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ZERODOL-SP</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>FND082504</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>03/2028</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="E157" t="n">
+        <v>80</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>10</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Strip of 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
           <t>ZINCOVIT TAB</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B158" t="inlineStr">
         <is>
           <t>ZVT25220</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>02/2027</t>
         </is>
       </c>
-      <c r="D156" t="n">
+      <c r="D158" t="n">
         <v>7.179</v>
       </c>
-      <c r="E156" t="n">
+      <c r="E158" t="n">
         <v>150</v>
       </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>Strip</t>
-        </is>
-      </c>
-      <c r="G156" t="n">
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Strip</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
         <v>15</v>
       </c>
-      <c r="H156" t="inlineStr">
+      <c r="H158" t="inlineStr">
         <is>
           <t>Strip of 15</t>
         </is>

</xml_diff>